<commit_message>
feat: finalize Phase 2 backend and documentation updates
</commit_message>
<xml_diff>
--- a/Product_Backlog.xlsx
+++ b/Product_Backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/22d7e69cf568a3bc/Documents/PythonProject/Final Project/FinalProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51CDE176-E1EA-48AB-9B5B-23C0CBECDFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{65D1735A-8D77-471C-AB7A-2322DB201657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72" yWindow="348" windowWidth="11448" windowHeight="7860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9048" yWindow="1824" windowWidth="11448" windowHeight="7860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="22">
   <si>
     <t>ITSC-3155 Software Engineering</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>Documentation and Training</t>
+  </si>
+  <si>
+    <t>Restaurant Staff Management</t>
   </si>
 </sst>
 </file>
@@ -438,6 +441,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -670,12 +674,24 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="2">
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
@@ -698,6 +714,8 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup fitToHeight="0" pageOrder="overThenDown" orientation="landscape" cellComments="atEnd"/>
 </worksheet>
 </file>
</xml_diff>